<commit_message>
updated arr values and churn percent in requirements catalog
</commit_message>
<xml_diff>
--- a/Requirements-Analysis/Requirements-Catalog-Tiimo.xlsx
+++ b/Requirements-Analysis/Requirements-Catalog-Tiimo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chitrangidoshi/Documents/Buisness Analyst/Case Study/Tiimo/Requirement Analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chitrangidoshi/Documents/Buisness Analyst/Case Study/Tiimo/github repo/Tiimo-Case-Study/Requirements-Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AE043B5-FA6B-1A42-A628-1D71820E8C3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B62FFA17-D11B-AE4A-BECA-4993BDC706C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -482,9 +482,6 @@
     <t>Achieve 70% Routines adoption, rating &gt;4.5 post-MVP</t>
   </si>
   <si>
-    <t>Reduce iPhone churn 20% via Routines MVP</t>
-  </si>
-  <si>
     <t>Product Managers, Data Analytics Team</t>
   </si>
   <si>
@@ -593,10 +590,13 @@
     <t>faq's in the app and website, train support team</t>
   </si>
   <si>
-    <t>Product needs Routines fit post-AI, more than $75k ROI</t>
-  </si>
-  <si>
     <t>Dev needs reusable timer engine for 4 sprint feasibility</t>
+  </si>
+  <si>
+    <t>Reduce iPhone churn 13.5% via Routines MVP</t>
+  </si>
+  <si>
+    <t>Product needs Routines fit post-AI,  $105k ROI</t>
   </si>
 </sst>
 </file>
@@ -604,7 +604,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -957,6 +957,18 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -980,18 +992,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1229,21 +1229,21 @@
   <sheetData>
     <row r="1" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="2" spans="1:18" ht="35.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="18" t="s">
-        <v>177</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
+      <c r="A2" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
     </row>
     <row r="3" spans="1:18" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
@@ -1323,34 +1323,34 @@
       <c r="A11" s="12"/>
     </row>
     <row r="12" spans="1:18" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="21"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="22" t="s">
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="H12" s="23"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="20" t="s">
+      <c r="H12" s="27"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="K12" s="25"/>
-      <c r="L12" s="20" t="s">
+      <c r="K12" s="29"/>
+      <c r="L12" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="M12" s="25"/>
-      <c r="N12" s="27" t="s">
+      <c r="M12" s="29"/>
+      <c r="N12" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="O12" s="28"/>
-      <c r="P12" s="28"/>
-      <c r="Q12" s="28"/>
-      <c r="R12" s="29"/>
+      <c r="O12" s="20"/>
+      <c r="P12" s="20"/>
+      <c r="Q12" s="20"/>
+      <c r="R12" s="21"/>
     </row>
     <row r="13" spans="1:18" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A13" s="15" t="s">
@@ -1440,7 +1440,7 @@
         <v>43</v>
       </c>
       <c r="K14" s="16" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L14" s="16" t="s">
         <v>38</v>
@@ -1448,20 +1448,20 @@
       <c r="M14" s="16">
         <v>1</v>
       </c>
-      <c r="N14" s="26">
+      <c r="N14" s="18">
         <v>10</v>
       </c>
-      <c r="O14" s="26">
+      <c r="O14" s="18">
         <v>10</v>
       </c>
-      <c r="P14" s="26">
+      <c r="P14" s="18">
         <v>0.9</v>
       </c>
-      <c r="Q14" s="26">
+      <c r="Q14" s="18">
         <v>1.5</v>
       </c>
-      <c r="R14" s="26">
-        <f>(N14*O14*P14)/Q14</f>
+      <c r="R14" s="18">
+        <f t="shared" ref="R14:R36" si="0">(N14*O14*P14)/Q14</f>
         <v>60</v>
       </c>
     </row>
@@ -1482,7 +1482,7 @@
         <v>35</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G15" s="16" t="s">
         <v>58</v>
@@ -1503,20 +1503,20 @@
       <c r="M15" s="16">
         <v>1</v>
       </c>
-      <c r="N15" s="26">
+      <c r="N15" s="18">
         <v>10</v>
       </c>
-      <c r="O15" s="26">
+      <c r="O15" s="18">
         <v>10</v>
       </c>
-      <c r="P15" s="26">
+      <c r="P15" s="18">
         <v>0.9</v>
       </c>
-      <c r="Q15" s="26">
+      <c r="Q15" s="18">
         <v>1.5</v>
       </c>
-      <c r="R15" s="26">
-        <f>(N15*O15*P15)/Q15</f>
+      <c r="R15" s="18">
+        <f t="shared" si="0"/>
         <v>60</v>
       </c>
     </row>
@@ -1540,7 +1540,7 @@
         <v>123</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H16" s="16" t="s">
         <v>37</v>
@@ -1560,20 +1560,20 @@
       <c r="M16" s="16">
         <v>1</v>
       </c>
-      <c r="N16" s="26">
+      <c r="N16" s="18">
         <v>10</v>
       </c>
-      <c r="O16" s="26">
+      <c r="O16" s="18">
         <v>10</v>
       </c>
-      <c r="P16" s="26">
+      <c r="P16" s="18">
         <v>0.9</v>
       </c>
-      <c r="Q16" s="26">
+      <c r="Q16" s="18">
         <v>1.5</v>
       </c>
-      <c r="R16" s="26">
-        <f>(N16*O16*P16)/Q16</f>
+      <c r="R16" s="18">
+        <f t="shared" si="0"/>
         <v>60</v>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
         <v>65</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>46</v>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="J17" s="16"/>
       <c r="K17" s="16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L17" s="16" t="s">
         <v>52</v>
@@ -1615,32 +1615,32 @@
       <c r="M17" s="16">
         <v>1</v>
       </c>
-      <c r="N17" s="26">
+      <c r="N17" s="18">
         <v>9</v>
       </c>
-      <c r="O17" s="26">
+      <c r="O17" s="18">
         <v>8</v>
       </c>
-      <c r="P17" s="26">
+      <c r="P17" s="18">
         <v>0.8</v>
       </c>
-      <c r="Q17" s="26">
+      <c r="Q17" s="18">
         <v>1</v>
       </c>
-      <c r="R17" s="26">
-        <f>(N17*O17*P17)/Q17</f>
+      <c r="R17" s="18">
+        <f t="shared" si="0"/>
         <v>57.6</v>
       </c>
     </row>
     <row r="18" spans="1:18" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B18" s="16" t="s">
         <v>103</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D18" s="16" t="s">
         <v>96</v>
@@ -1672,20 +1672,20 @@
       <c r="M18" s="16">
         <v>1</v>
       </c>
-      <c r="N18" s="26">
+      <c r="N18" s="18">
         <v>9</v>
       </c>
-      <c r="O18" s="26">
+      <c r="O18" s="18">
         <v>8</v>
       </c>
-      <c r="P18" s="26">
+      <c r="P18" s="18">
         <v>0.8</v>
       </c>
-      <c r="Q18" s="26">
+      <c r="Q18" s="18">
         <v>1</v>
       </c>
-      <c r="R18" s="26">
-        <f>(N18*O18*P18)/Q18</f>
+      <c r="R18" s="18">
+        <f t="shared" si="0"/>
         <v>57.6</v>
       </c>
     </row>
@@ -1694,10 +1694,10 @@
         <v>95</v>
       </c>
       <c r="B19" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="C19" s="16" t="s">
         <v>170</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>171</v>
       </c>
       <c r="D19" s="16" t="s">
         <v>96</v>
@@ -1706,7 +1706,7 @@
         <v>35</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G19" s="16" t="s">
         <v>58</v>
@@ -1715,7 +1715,7 @@
         <v>37</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="J19" s="16" t="s">
         <v>63</v>
@@ -1729,20 +1729,20 @@
       <c r="M19" s="16">
         <v>1</v>
       </c>
-      <c r="N19" s="26">
+      <c r="N19" s="18">
         <v>10</v>
       </c>
-      <c r="O19" s="26">
+      <c r="O19" s="18">
         <v>9</v>
       </c>
-      <c r="P19" s="26">
+      <c r="P19" s="18">
         <v>0.9</v>
       </c>
-      <c r="Q19" s="26">
+      <c r="Q19" s="18">
         <v>1.5</v>
       </c>
-      <c r="R19" s="26">
-        <f>(N19*O19*P19)/Q19</f>
+      <c r="R19" s="18">
+        <f t="shared" si="0"/>
         <v>54</v>
       </c>
     </row>
@@ -1784,20 +1784,20 @@
       <c r="M20" s="16">
         <v>1</v>
       </c>
-      <c r="N20" s="26">
+      <c r="N20" s="18">
         <v>8</v>
       </c>
-      <c r="O20" s="26">
+      <c r="O20" s="18">
         <v>8</v>
       </c>
-      <c r="P20" s="26">
+      <c r="P20" s="18">
         <v>0.8</v>
       </c>
-      <c r="Q20" s="26">
+      <c r="Q20" s="18">
         <v>1</v>
       </c>
-      <c r="R20" s="26">
-        <f>(N20*O20*P20)/Q20</f>
+      <c r="R20" s="18">
+        <f t="shared" si="0"/>
         <v>51.2</v>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
         <v>35</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>58</v>
@@ -1841,20 +1841,20 @@
       <c r="M21" s="16">
         <v>1</v>
       </c>
-      <c r="N21" s="26">
+      <c r="N21" s="18">
         <v>9</v>
       </c>
-      <c r="O21" s="26">
+      <c r="O21" s="18">
         <v>9</v>
       </c>
-      <c r="P21" s="26">
+      <c r="P21" s="18">
         <v>0.9</v>
       </c>
-      <c r="Q21" s="26">
+      <c r="Q21" s="18">
         <v>1.5</v>
       </c>
-      <c r="R21" s="26">
-        <f>(N21*O21*P21)/Q21</f>
+      <c r="R21" s="18">
+        <f t="shared" si="0"/>
         <v>48.6</v>
       </c>
     </row>
@@ -1863,10 +1863,10 @@
         <v>97</v>
       </c>
       <c r="B22" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="C22" s="16" t="s">
         <v>174</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>175</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>96</v>
@@ -1875,7 +1875,7 @@
         <v>35</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G22" s="16" t="s">
         <v>58</v>
@@ -1884,7 +1884,7 @@
         <v>37</v>
       </c>
       <c r="I22" s="16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>63</v>
@@ -1898,20 +1898,20 @@
       <c r="M22" s="16">
         <v>1</v>
       </c>
-      <c r="N22" s="26">
+      <c r="N22" s="18">
         <v>10</v>
       </c>
-      <c r="O22" s="26">
+      <c r="O22" s="18">
         <v>9</v>
       </c>
-      <c r="P22" s="26">
+      <c r="P22" s="18">
         <v>0.8</v>
       </c>
-      <c r="Q22" s="26">
+      <c r="Q22" s="18">
         <v>1.5</v>
       </c>
-      <c r="R22" s="26">
-        <f>(N22*O22*P22)/Q22</f>
+      <c r="R22" s="18">
+        <f t="shared" si="0"/>
         <v>48</v>
       </c>
     </row>
@@ -1920,10 +1920,10 @@
         <v>105</v>
       </c>
       <c r="B23" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="C23" s="16" t="s">
         <v>182</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>183</v>
       </c>
       <c r="D23" s="16" t="s">
         <v>106</v>
@@ -1932,7 +1932,7 @@
         <v>94</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G23" s="16" t="s">
         <v>58</v>
@@ -1951,20 +1951,20 @@
       <c r="M23" s="16">
         <v>1</v>
       </c>
-      <c r="N23" s="26">
+      <c r="N23" s="18">
         <v>5</v>
       </c>
-      <c r="O23" s="26">
+      <c r="O23" s="18">
         <v>6</v>
       </c>
-      <c r="P23" s="26">
+      <c r="P23" s="18">
         <v>0.7</v>
       </c>
-      <c r="Q23" s="26">
+      <c r="Q23" s="18">
         <v>0.5</v>
       </c>
-      <c r="R23" s="26">
-        <f>(N23*O23*P23)/Q23</f>
+      <c r="R23" s="18">
+        <f t="shared" si="0"/>
         <v>42</v>
       </c>
     </row>
@@ -1976,7 +1976,7 @@
         <v>57</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D24" s="16" t="s">
         <v>46</v>
@@ -2000,7 +2000,7 @@
         <v>59</v>
       </c>
       <c r="K24" s="16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="L24" s="16" t="s">
         <v>38</v>
@@ -2008,20 +2008,20 @@
       <c r="M24" s="16">
         <v>1</v>
       </c>
-      <c r="N24" s="26">
+      <c r="N24" s="18">
         <v>8</v>
       </c>
-      <c r="O24" s="26">
+      <c r="O24" s="18">
         <v>9</v>
       </c>
-      <c r="P24" s="26">
+      <c r="P24" s="18">
         <v>0.8</v>
       </c>
-      <c r="Q24" s="26">
+      <c r="Q24" s="18">
         <v>1.5</v>
       </c>
-      <c r="R24" s="26">
-        <f>(N24*O24*P24)/Q24</f>
+      <c r="R24" s="18">
+        <f t="shared" si="0"/>
         <v>38.4</v>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
         <v>142</v>
       </c>
       <c r="I25" s="16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J25" s="16" t="s">
         <v>47</v>
@@ -2063,20 +2063,20 @@
       <c r="M25" s="16">
         <v>1</v>
       </c>
-      <c r="N25" s="26">
+      <c r="N25" s="18">
         <v>10</v>
       </c>
-      <c r="O25" s="26">
+      <c r="O25" s="18">
         <v>10</v>
       </c>
-      <c r="P25" s="26">
+      <c r="P25" s="18">
         <v>0.9</v>
       </c>
-      <c r="Q25" s="26">
+      <c r="Q25" s="18">
         <v>2.5</v>
       </c>
-      <c r="R25" s="26">
-        <f>(N25*O25*P25)/Q25</f>
+      <c r="R25" s="18">
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
     </row>
@@ -2112,7 +2112,7 @@
         <v>63</v>
       </c>
       <c r="K26" s="16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L26" s="16" t="s">
         <v>38</v>
@@ -2120,20 +2120,20 @@
       <c r="M26" s="16">
         <v>1</v>
       </c>
-      <c r="N26" s="26">
+      <c r="N26" s="18">
         <v>7</v>
       </c>
-      <c r="O26" s="26">
+      <c r="O26" s="18">
         <v>7</v>
       </c>
-      <c r="P26" s="26">
+      <c r="P26" s="18">
         <v>0.7</v>
       </c>
-      <c r="Q26" s="26">
+      <c r="Q26" s="18">
         <v>1</v>
       </c>
-      <c r="R26" s="26">
-        <f>(N26*O26*P26)/Q26</f>
+      <c r="R26" s="18">
+        <f t="shared" si="0"/>
         <v>34.299999999999997</v>
       </c>
     </row>
@@ -2142,7 +2142,7 @@
         <v>53</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>129</v>
@@ -2169,7 +2169,7 @@
         <v>55</v>
       </c>
       <c r="K27" s="16" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="L27" s="16" t="s">
         <v>38</v>
@@ -2177,20 +2177,20 @@
       <c r="M27" s="16">
         <v>1</v>
       </c>
-      <c r="N27" s="26">
+      <c r="N27" s="18">
         <v>9</v>
       </c>
-      <c r="O27" s="26">
+      <c r="O27" s="18">
         <v>9</v>
       </c>
-      <c r="P27" s="26">
+      <c r="P27" s="18">
         <v>0.8</v>
       </c>
-      <c r="Q27" s="26">
+      <c r="Q27" s="18">
         <v>2</v>
       </c>
-      <c r="R27" s="26">
-        <f>(N27*O27*P27)/Q27</f>
+      <c r="R27" s="18">
+        <f t="shared" si="0"/>
         <v>32.4</v>
       </c>
     </row>
@@ -2202,7 +2202,7 @@
         <v>84</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D28" s="16" t="s">
         <v>74</v>
@@ -2234,20 +2234,20 @@
       <c r="M28" s="16">
         <v>1</v>
       </c>
-      <c r="N28" s="26">
+      <c r="N28" s="18">
         <v>9</v>
       </c>
-      <c r="O28" s="26">
+      <c r="O28" s="18">
         <v>9</v>
       </c>
-      <c r="P28" s="26">
+      <c r="P28" s="18">
         <v>0.8</v>
       </c>
-      <c r="Q28" s="26">
+      <c r="Q28" s="18">
         <v>2</v>
       </c>
-      <c r="R28" s="26">
-        <f>(N28*O28*P28)/Q28</f>
+      <c r="R28" s="18">
+        <f t="shared" si="0"/>
         <v>32.4</v>
       </c>
     </row>
@@ -2256,10 +2256,10 @@
         <v>91</v>
       </c>
       <c r="B29" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="C29" s="16" t="s">
         <v>167</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>168</v>
       </c>
       <c r="D29" s="16" t="s">
         <v>74</v>
@@ -2289,20 +2289,20 @@
       <c r="M29" s="16">
         <v>1</v>
       </c>
-      <c r="N29" s="26">
+      <c r="N29" s="18">
         <v>9</v>
       </c>
-      <c r="O29" s="26">
+      <c r="O29" s="18">
         <v>9</v>
       </c>
-      <c r="P29" s="26">
+      <c r="P29" s="18">
         <v>0.75</v>
       </c>
-      <c r="Q29" s="26">
+      <c r="Q29" s="18">
         <v>2</v>
       </c>
-      <c r="R29" s="26">
-        <f>(N29*O29*P29)/Q29</f>
+      <c r="R29" s="18">
+        <f t="shared" si="0"/>
         <v>30.375</v>
       </c>
     </row>
@@ -2314,7 +2314,7 @@
         <v>33</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>148</v>
+        <v>185</v>
       </c>
       <c r="D30" s="16" t="s">
         <v>34</v>
@@ -2344,20 +2344,20 @@
       <c r="M30" s="16">
         <v>1</v>
       </c>
-      <c r="N30" s="26">
+      <c r="N30" s="18">
         <v>10</v>
       </c>
-      <c r="O30" s="26">
+      <c r="O30" s="18">
         <v>10</v>
       </c>
-      <c r="P30" s="26">
+      <c r="P30" s="18">
         <v>0.9</v>
       </c>
-      <c r="Q30" s="26">
+      <c r="Q30" s="18">
         <v>3</v>
       </c>
-      <c r="R30" s="26">
-        <f>(N30*O30*P30)/Q30</f>
+      <c r="R30" s="18">
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
         <v>37</v>
       </c>
       <c r="I31" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J31" s="16" t="s">
         <v>86</v>
@@ -2399,20 +2399,20 @@
       <c r="M31" s="16">
         <v>1</v>
       </c>
-      <c r="N31" s="26">
+      <c r="N31" s="18">
         <v>7</v>
       </c>
-      <c r="O31" s="26">
+      <c r="O31" s="18">
         <v>6</v>
       </c>
-      <c r="P31" s="26">
+      <c r="P31" s="18">
         <v>0.7</v>
       </c>
-      <c r="Q31" s="26">
+      <c r="Q31" s="18">
         <v>1</v>
       </c>
-      <c r="R31" s="26">
-        <f>(N31*O31*P31)/Q31</f>
+      <c r="R31" s="18">
+        <f t="shared" si="0"/>
         <v>29.4</v>
       </c>
     </row>
@@ -2442,7 +2442,7 @@
         <v>37</v>
       </c>
       <c r="I32" s="16" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J32" s="16" t="s">
         <v>89</v>
@@ -2456,20 +2456,20 @@
       <c r="M32" s="16">
         <v>1</v>
       </c>
-      <c r="N32" s="26">
+      <c r="N32" s="18">
         <v>9</v>
       </c>
-      <c r="O32" s="26">
+      <c r="O32" s="18">
         <v>8</v>
       </c>
-      <c r="P32" s="26">
+      <c r="P32" s="18">
         <v>0.8</v>
       </c>
-      <c r="Q32" s="26">
+      <c r="Q32" s="18">
         <v>2</v>
       </c>
-      <c r="R32" s="26">
-        <f>(N32*O32*P32)/Q32</f>
+      <c r="R32" s="18">
+        <f t="shared" si="0"/>
         <v>28.8</v>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
         <v>41</v>
       </c>
       <c r="F33" s="16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G33" s="16" t="s">
         <v>144</v>
@@ -2499,11 +2499,11 @@
         <v>144</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J33" s="16"/>
       <c r="K33" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L33" s="16" t="s">
         <v>38</v>
@@ -2511,20 +2511,20 @@
       <c r="M33" s="16">
         <v>1</v>
       </c>
-      <c r="N33" s="26">
+      <c r="N33" s="18">
         <v>6</v>
       </c>
-      <c r="O33" s="26">
+      <c r="O33" s="18">
         <v>8</v>
       </c>
-      <c r="P33" s="26">
+      <c r="P33" s="18">
         <v>0.7</v>
       </c>
-      <c r="Q33" s="26">
+      <c r="Q33" s="18">
         <v>1.5</v>
       </c>
-      <c r="R33" s="26">
-        <f>(N33*O33*P33)/Q33</f>
+      <c r="R33" s="18">
+        <f t="shared" si="0"/>
         <v>22.399999999999995</v>
       </c>
     </row>
@@ -2545,7 +2545,7 @@
         <v>41</v>
       </c>
       <c r="F34" s="16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G34" s="16" t="s">
         <v>145</v>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="J34" s="16"/>
       <c r="K34" s="16" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L34" s="16" t="s">
         <v>38</v>
@@ -2566,20 +2566,20 @@
       <c r="M34" s="16">
         <v>1</v>
       </c>
-      <c r="N34" s="26">
+      <c r="N34" s="18">
         <v>7</v>
       </c>
-      <c r="O34" s="26">
+      <c r="O34" s="18">
         <v>9</v>
       </c>
-      <c r="P34" s="26">
+      <c r="P34" s="18">
         <v>0.7</v>
       </c>
-      <c r="Q34" s="26">
+      <c r="Q34" s="18">
         <v>2</v>
       </c>
-      <c r="R34" s="26">
-        <f>(N34*O34*P34)/Q34</f>
+      <c r="R34" s="18">
+        <f t="shared" si="0"/>
         <v>22.049999999999997</v>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
         <v>42</v>
       </c>
       <c r="I35" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J35" s="16"/>
       <c r="K35" s="16" t="s">
@@ -2621,20 +2621,20 @@
       <c r="M35" s="16">
         <v>1</v>
       </c>
-      <c r="N35" s="26">
+      <c r="N35" s="18">
         <v>10</v>
       </c>
-      <c r="O35" s="26">
+      <c r="O35" s="18">
         <v>10</v>
       </c>
-      <c r="P35" s="26">
+      <c r="P35" s="18">
         <v>0.8</v>
       </c>
-      <c r="Q35" s="26">
+      <c r="Q35" s="18">
         <v>4</v>
       </c>
-      <c r="R35" s="26">
-        <f>(N35*O35*P35)/Q35</f>
+      <c r="R35" s="18">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
@@ -2643,7 +2643,7 @@
         <v>48</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>49</v>
@@ -2664,7 +2664,7 @@
         <v>42</v>
       </c>
       <c r="I36" s="16" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J36" s="16" t="s">
         <v>51</v>
@@ -2676,20 +2676,20 @@
       <c r="M36" s="16">
         <v>1</v>
       </c>
-      <c r="N36" s="26">
+      <c r="N36" s="18">
         <v>8</v>
       </c>
-      <c r="O36" s="26">
+      <c r="O36" s="18">
         <v>9</v>
       </c>
-      <c r="P36" s="26">
+      <c r="P36" s="18">
         <v>0.8</v>
       </c>
-      <c r="Q36" s="26">
+      <c r="Q36" s="18">
         <v>4</v>
       </c>
-      <c r="R36" s="26">
-        <f>(N36*O36*P36)/Q36</f>
+      <c r="R36" s="18">
+        <f t="shared" si="0"/>
         <v>14.4</v>
       </c>
     </row>

</xml_diff>